<commit_message>
Aged-FG push email 29-Oct in the 26-Oct sent format
Progress vs 26-Oct (base restated with the 30-Sep invoices), stock by
plant with actions, SKUs to push with a 'sold since 26-Oct' column, and
the SKUs where nothing moved. Attachment gains the same column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SVVKmwQKKV189dev92iFna
</commit_message>
<xml_diff>
--- a/reports/FG-Over-30-Days-2026-10-29.xlsx
+++ b/reports/FG-Over-30-Days-2026-10-29.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Over 30 days" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Over 30 days'!$A$4:$J$54</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Over 30 days'!$A$4:$K$54</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="88">
   <si>
     <t xml:space="preserve">Finished stock over 30 days, by plant (MT) - 29-Oct-2026</t>
   </si>
@@ -53,6 +53,12 @@
     <t xml:space="preserve">Over 60 days</t>
   </si>
   <si>
+    <t xml:space="preserve">Over 30 days on 26-Oct (restated, system)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoiced from it since</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hyderabad</t>
   </si>
   <si>
@@ -65,15 +71,18 @@
     <t xml:space="preserve">West</t>
   </si>
   <si>
+    <t xml:space="preserve">Tapi</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lepakshi</t>
   </si>
   <si>
-    <t xml:space="preserve">Tapi</t>
-  </si>
-  <si>
     <t xml:space="preserve">Total</t>
   </si>
   <si>
+    <t xml:space="preserve">Columns I-J are whole-plant system figures from the database (including SKUs whose aged stock sold out); D-H add up the "Over 30 days" sheet.</t>
+  </si>
+  <si>
     <t xml:space="preserve">JSW Pipes &amp; Tubes - finished stock older than 30 days, by plant and SKU (reconciled to plant FG statements)</t>
   </si>
   <si>
@@ -104,6 +113,9 @@
     <t xml:space="preserve">Total FG of this SKU at the plant (MT)</t>
   </si>
   <si>
+    <t xml:space="preserve">Sold since 26-Oct (MT)</t>
+  </si>
+  <si>
     <t xml:space="preserve">P1: oldest batch over 90 days</t>
   </si>
   <si>
@@ -188,6 +200,9 @@
     <t xml:space="preserve">CHS 15 NB x 2.5</t>
   </si>
   <si>
+    <t xml:space="preserve">new</t>
+  </si>
+  <si>
     <t xml:space="preserve">CHS 15 NB x 2</t>
   </si>
   <si>
@@ -224,33 +239,33 @@
     <t xml:space="preserve">RHS 50x25 x 1.6</t>
   </si>
   <si>
+    <t xml:space="preserve">SHS 50x50 x 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SHS 150x150 x 2.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RHS 145x82 x 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RHS 145x82 x 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SHS 100x100 x 5</t>
+  </si>
+  <si>
     <t xml:space="preserve">SHS 72x72 x 5</t>
   </si>
   <si>
     <t xml:space="preserve">SHS 72x72 x 2.5</t>
   </si>
   <si>
-    <t xml:space="preserve">SHS 100x100 x 5</t>
-  </si>
-  <si>
     <t xml:space="preserve">RHS 96x48 x 2.5</t>
   </si>
   <si>
     <t xml:space="preserve">SHS 100x100 x 2.5</t>
   </si>
   <si>
-    <t xml:space="preserve">SHS 50x50 x 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SHS 150x150 x 2.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RHS 145x82 x 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RHS 145x82 x 4</t>
-  </si>
-  <si>
     <t xml:space="preserve">Total (follows the filter)</t>
   </si>
   <si>
@@ -264,6 +279,9 @@
   </si>
   <si>
     <t xml:space="preserve">Thickness is grouped to 1.6 / 2 / 2.5 / 3 / 4 / 5 / 6 mm. Stock the plants hold but the system has no production record for is not aged and not listed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Sold since 26-Oct" = tonnes of that SKU's over-30-day stock of 26-Oct (system, restated with the 30-Sep invoices loaded on 29-Oct) invoiced since; 0.00 (red) = nothing moved; "new" = crossed 30 days this week. Not totalled: SKUs whose aged stock sold out are not listed.</t>
   </si>
   <si>
     <t xml:space="preserve">Sells to: Hyderabad and Lepakshi serve South distributors; NPMD and Tapi serve West. Use the filter arrows to pick a plant, region or priority.</t>
@@ -276,12 +294,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00;\-#,##0.00;\-"/>
     <numFmt numFmtId="166" formatCode="0"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -334,6 +353,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FF555555"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <i val="true"/>
       <sz val="9"/>
       <color rgb="FF555555"/>
@@ -343,13 +369,29 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="9"/>
-      <color rgb="FF555555"/>
+      <sz val="10"/>
+      <color rgb="FF9B1C1C"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <color rgb="FF8A5300"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1E6B34"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="9"/>
       <color rgb="FF555555"/>
       <name val="Arial"/>
@@ -444,7 +486,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -485,6 +527,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -501,6 +547,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -509,11 +559,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -526,7 +580,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -574,6 +628,30 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF1E6B34"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF8A5300"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9B1C1C"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <colors>
     <indexedColors>
@@ -586,9 +664,9 @@
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF1E6B34"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF8A5300"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFC0C0C0"/>
@@ -629,7 +707,7 @@
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF9B1C1C"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
@@ -822,7 +900,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -830,6 +908,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -837,7 +917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -862,13 +942,19 @@
       <c r="H3" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="I3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" s="5" t="n">
         <f aca="false">COUNTIF('Over 30 days'!$B$5:$B$54,A4)</f>
@@ -894,13 +980,19 @@
         <f aca="false">F4+G4</f>
         <v>220.189008018403</v>
       </c>
+      <c r="I4" s="4" t="n">
+        <v>336.369498987128</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>11.0970854980678</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">COUNTIF('Over 30 days'!$B$5:$B$54,A5)</f>
@@ -926,25 +1018,31 @@
         <f aca="false">F5+G5</f>
         <v>0</v>
       </c>
+      <c r="I5" s="4" t="n">
+        <v>131.928534368</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>28.13654368</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">COUNTIF('Over 30 days'!$B$5:$B$54,A6)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D6" s="4" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$54,A6,'Over 30 days'!$E$5:$E$54)</f>
-        <v>80.1</v>
+        <v>24.6600492700294</v>
       </c>
       <c r="E6" s="4" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$54,A6,'Over 30 days'!$F$5:$F$54)</f>
-        <v>80.1</v>
+        <v>24.6600492700294</v>
       </c>
       <c r="F6" s="4" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$54,A6,'Over 30 days'!$G$5:$G$54)</f>
@@ -958,25 +1056,31 @@
         <f aca="false">F6+G6</f>
         <v>0</v>
       </c>
+      <c r="I6" s="4" t="n">
+        <v>19.7118372</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>6.562</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">COUNTIF('Over 30 days'!$B$5:$B$54,A7)</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D7" s="4" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$54,A7,'Over 30 days'!$E$5:$E$54)</f>
-        <v>24.6600492700294</v>
+        <v>80.1</v>
       </c>
       <c r="E7" s="4" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$54,A7,'Over 30 days'!$F$5:$F$54)</f>
-        <v>24.6600492700294</v>
+        <v>80.1</v>
       </c>
       <c r="F7" s="4" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$54,A7,'Over 30 days'!$G$5:$G$54)</f>
@@ -990,10 +1094,16 @@
         <f aca="false">F7+G7</f>
         <v>0</v>
       </c>
+      <c r="I7" s="4" t="n">
+        <v>62.1526841</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="7" t="n">
@@ -1019,6 +1129,19 @@
       <c r="H8" s="8" t="n">
         <f aca="false">SUM(H4:H7)</f>
         <v>220.189008018403</v>
+      </c>
+      <c r="I8" s="8" t="n">
+        <f aca="false">SUM(I4:I7)</f>
+        <v>550.162554655128</v>
+      </c>
+      <c r="J8" s="8" t="n">
+        <f aca="false">SUM(J4:J7)</f>
+        <v>45.7956291780678</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1037,7 +1160,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:J62"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -1048,62 +1171,66 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
-        <v>17</v>
+      <c r="A2" s="10" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="10" t="s">
+      <c r="A4" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="10" t="s">
+      <c r="D4" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="E4" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="F4" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="G4" s="11" t="s">
         <v>25</v>
       </c>
+      <c r="H4" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>27</v>
+      <c r="A5" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>31</v>
       </c>
       <c r="E5" s="3" t="n">
         <f aca="false">SUM(F5:H5)</f>
@@ -1118,25 +1245,28 @@
       <c r="H5" s="4" t="n">
         <v>29.0650131191129</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="I5" s="13" t="n">
         <v>114</v>
       </c>
       <c r="J5" s="4" t="n">
         <v>33.383</v>
       </c>
+      <c r="K5" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>28</v>
+      <c r="A6" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>32</v>
       </c>
       <c r="E6" s="3" t="n">
         <f aca="false">SUM(F6:H6)</f>
@@ -1151,25 +1281,28 @@
       <c r="H6" s="4" t="n">
         <v>27.325</v>
       </c>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="13" t="n">
         <v>128</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>27.325</v>
       </c>
+      <c r="K6" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>29</v>
+      <c r="A7" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>33</v>
       </c>
       <c r="E7" s="3" t="n">
         <f aca="false">SUM(F7:H7)</f>
@@ -1184,25 +1317,28 @@
       <c r="H7" s="4" t="n">
         <v>4.25865238176696</v>
       </c>
-      <c r="I7" s="12" t="n">
+      <c r="I7" s="13" t="n">
         <v>104</v>
       </c>
       <c r="J7" s="4" t="n">
         <v>25.549</v>
       </c>
+      <c r="K7" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="13" t="s">
+      <c r="A8" s="12" t="s">
         <v>30</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>34</v>
       </c>
       <c r="E8" s="3" t="n">
         <f aca="false">SUM(F8:H8)</f>
@@ -1217,25 +1353,28 @@
       <c r="H8" s="4" t="n">
         <v>20.8701170459605</v>
       </c>
-      <c r="I8" s="12" t="n">
+      <c r="I8" s="13" t="n">
         <v>111</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>25.051</v>
       </c>
+      <c r="K8" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>31</v>
+      <c r="A9" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>35</v>
       </c>
       <c r="E9" s="3" t="n">
         <f aca="false">SUM(F9:H9)</f>
@@ -1250,25 +1389,28 @@
       <c r="H9" s="4" t="n">
         <v>18.573</v>
       </c>
-      <c r="I9" s="12" t="n">
+      <c r="I9" s="13" t="n">
         <v>189</v>
       </c>
       <c r="J9" s="4" t="n">
         <v>18.573</v>
       </c>
+      <c r="K9" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>32</v>
+      <c r="A10" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>36</v>
       </c>
       <c r="E10" s="3" t="n">
         <f aca="false">SUM(F10:H10)</f>
@@ -1283,25 +1425,28 @@
       <c r="H10" s="4" t="n">
         <v>17.065</v>
       </c>
-      <c r="I10" s="12" t="n">
+      <c r="I10" s="13" t="n">
         <v>114</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>17.065</v>
       </c>
+      <c r="K10" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>33</v>
+      <c r="A11" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>37</v>
       </c>
       <c r="E11" s="3" t="n">
         <f aca="false">SUM(F11:H11)</f>
@@ -1316,25 +1461,28 @@
       <c r="H11" s="4" t="n">
         <v>15.096</v>
       </c>
-      <c r="I11" s="12" t="n">
+      <c r="I11" s="13" t="n">
         <v>113</v>
       </c>
       <c r="J11" s="4" t="n">
         <v>15.096</v>
       </c>
+      <c r="K11" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>34</v>
+      <c r="A12" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>38</v>
       </c>
       <c r="E12" s="3" t="n">
         <f aca="false">SUM(F12:H12)</f>
@@ -1349,25 +1497,28 @@
       <c r="H12" s="4" t="n">
         <v>12.48</v>
       </c>
-      <c r="I12" s="12" t="n">
+      <c r="I12" s="13" t="n">
         <v>127</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>12.48</v>
       </c>
+      <c r="K12" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>35</v>
+      <c r="A13" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>39</v>
       </c>
       <c r="E13" s="3" t="n">
         <f aca="false">SUM(F13:H13)</f>
@@ -1382,25 +1533,28 @@
       <c r="H13" s="4" t="n">
         <v>9.983</v>
       </c>
-      <c r="I13" s="12" t="n">
+      <c r="I13" s="13" t="n">
         <v>187</v>
       </c>
       <c r="J13" s="4" t="n">
         <v>9.983</v>
       </c>
+      <c r="K13" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>36</v>
+      <c r="A14" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>40</v>
       </c>
       <c r="E14" s="3" t="n">
         <f aca="false">SUM(F14:H14)</f>
@@ -1415,25 +1569,28 @@
       <c r="H14" s="4" t="n">
         <v>9.70464731636379</v>
       </c>
-      <c r="I14" s="12" t="n">
+      <c r="I14" s="13" t="n">
         <v>99</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>18.327</v>
       </c>
+      <c r="K14" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>37</v>
+      <c r="A15" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>41</v>
       </c>
       <c r="E15" s="3" t="n">
         <f aca="false">SUM(F15:H15)</f>
@@ -1448,25 +1605,28 @@
       <c r="H15" s="4" t="n">
         <v>9.52274105432948</v>
       </c>
-      <c r="I15" s="12" t="n">
+      <c r="I15" s="13" t="n">
         <v>91</v>
       </c>
       <c r="J15" s="4" t="n">
         <v>12.496</v>
       </c>
+      <c r="K15" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>38</v>
+      <c r="A16" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>42</v>
       </c>
       <c r="E16" s="3" t="n">
         <f aca="false">SUM(F16:H16)</f>
@@ -1481,25 +1641,28 @@
       <c r="H16" s="4" t="n">
         <v>9.126</v>
       </c>
-      <c r="I16" s="12" t="n">
+      <c r="I16" s="13" t="n">
         <v>123</v>
       </c>
       <c r="J16" s="4" t="n">
         <v>9.126</v>
       </c>
+      <c r="K16" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>39</v>
+      <c r="A17" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>43</v>
       </c>
       <c r="E17" s="3" t="n">
         <f aca="false">SUM(F17:H17)</f>
@@ -1514,25 +1677,28 @@
       <c r="H17" s="4" t="n">
         <v>8.76362094261573</v>
       </c>
-      <c r="I17" s="12" t="n">
+      <c r="I17" s="13" t="n">
         <v>136</v>
       </c>
       <c r="J17" s="4" t="n">
         <v>10.119</v>
       </c>
+      <c r="K17" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>40</v>
+      <c r="A18" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>44</v>
       </c>
       <c r="E18" s="3" t="n">
         <f aca="false">SUM(F18:H18)</f>
@@ -1547,25 +1713,28 @@
       <c r="H18" s="4" t="n">
         <v>5.509</v>
       </c>
-      <c r="I18" s="12" t="n">
+      <c r="I18" s="13" t="n">
         <v>128</v>
       </c>
       <c r="J18" s="4" t="n">
         <v>5.509</v>
       </c>
+      <c r="K18" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>41</v>
+      <c r="A19" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>45</v>
       </c>
       <c r="E19" s="3" t="n">
         <f aca="false">SUM(F19:H19)</f>
@@ -1580,25 +1749,28 @@
       <c r="H19" s="4" t="n">
         <v>2.31970749760539</v>
       </c>
-      <c r="I19" s="12" t="n">
+      <c r="I19" s="13" t="n">
         <v>99</v>
       </c>
       <c r="J19" s="4" t="n">
         <v>8.571</v>
       </c>
+      <c r="K19" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>42</v>
+      <c r="A20" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>46</v>
       </c>
       <c r="E20" s="3" t="n">
         <f aca="false">SUM(F20:H20)</f>
@@ -1613,25 +1785,28 @@
       <c r="H20" s="4" t="n">
         <v>2.182</v>
       </c>
-      <c r="I20" s="12" t="n">
+      <c r="I20" s="13" t="n">
         <v>122</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>2.182</v>
       </c>
+      <c r="K20" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D21" s="13" t="s">
-        <v>43</v>
+      <c r="A21" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>47</v>
       </c>
       <c r="E21" s="3" t="n">
         <f aca="false">SUM(F21:H21)</f>
@@ -1646,25 +1821,28 @@
       <c r="H21" s="4" t="n">
         <v>2.13250866064806</v>
       </c>
-      <c r="I21" s="12" t="n">
+      <c r="I21" s="13" t="n">
         <v>115</v>
       </c>
       <c r="J21" s="4" t="n">
         <v>3.03</v>
       </c>
+      <c r="K21" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" s="13" t="s">
-        <v>44</v>
+      <c r="A22" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>48</v>
       </c>
       <c r="E22" s="3" t="n">
         <f aca="false">SUM(F22:H22)</f>
@@ -1679,25 +1857,28 @@
       <c r="H22" s="4" t="n">
         <v>1.749</v>
       </c>
-      <c r="I22" s="12" t="n">
+      <c r="I22" s="13" t="n">
         <v>97</v>
       </c>
       <c r="J22" s="4" t="n">
         <v>1.749</v>
       </c>
+      <c r="K22" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" s="13" t="s">
-        <v>46</v>
+      <c r="A23" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>50</v>
       </c>
       <c r="E23" s="3" t="n">
         <f aca="false">SUM(F23:H23)</f>
@@ -1712,25 +1893,28 @@
       <c r="H23" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I23" s="12" t="n">
+      <c r="I23" s="13" t="n">
         <v>71</v>
       </c>
       <c r="J23" s="4" t="n">
         <v>7.702</v>
       </c>
+      <c r="K23" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D24" s="13" t="s">
-        <v>47</v>
+      <c r="A24" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>51</v>
       </c>
       <c r="E24" s="3" t="n">
         <f aca="false">SUM(F24:H24)</f>
@@ -1745,25 +1929,28 @@
       <c r="H24" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I24" s="12" t="n">
+      <c r="I24" s="13" t="n">
         <v>68</v>
       </c>
       <c r="J24" s="4" t="n">
         <v>6.762</v>
       </c>
+      <c r="K24" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="13" t="s">
-        <v>49</v>
+      <c r="A25" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="14" t="s">
+        <v>53</v>
       </c>
       <c r="E25" s="3" t="n">
         <f aca="false">SUM(F25:H25)</f>
@@ -1778,25 +1965,28 @@
       <c r="H25" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I25" s="12" t="n">
+      <c r="I25" s="13" t="n">
         <v>40</v>
       </c>
       <c r="J25" s="4" t="n">
         <v>13.237</v>
       </c>
+      <c r="K25" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D26" s="13" t="s">
-        <v>50</v>
+      <c r="A26" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>54</v>
       </c>
       <c r="E26" s="3" t="n">
         <f aca="false">SUM(F26:H26)</f>
@@ -1811,25 +2001,28 @@
       <c r="H26" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I26" s="12" t="n">
+      <c r="I26" s="13" t="n">
         <v>48</v>
       </c>
       <c r="J26" s="4" t="n">
         <v>11.674</v>
       </c>
+      <c r="K26" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B27" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" s="13" t="s">
-        <v>51</v>
+      <c r="A27" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="14" t="s">
+        <v>55</v>
       </c>
       <c r="E27" s="3" t="n">
         <f aca="false">SUM(F27:H27)</f>
@@ -1844,25 +2037,28 @@
       <c r="H27" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I27" s="12" t="n">
+      <c r="I27" s="13" t="n">
         <v>45</v>
       </c>
       <c r="J27" s="4" t="n">
         <v>10.076</v>
       </c>
+      <c r="K27" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="13" t="s">
+      <c r="A28" s="17" t="s">
         <v>52</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>56</v>
       </c>
       <c r="E28" s="3" t="n">
         <f aca="false">SUM(F28:H28)</f>
@@ -1877,25 +2073,28 @@
       <c r="H28" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I28" s="12" t="n">
+      <c r="I28" s="13" t="n">
         <v>41</v>
       </c>
       <c r="J28" s="4" t="n">
         <v>11.431</v>
       </c>
+      <c r="K28" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D29" s="13" t="s">
-        <v>53</v>
+      <c r="A29" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>57</v>
       </c>
       <c r="E29" s="3" t="n">
         <f aca="false">SUM(F29:H29)</f>
@@ -1910,25 +2109,28 @@
       <c r="H29" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I29" s="12" t="n">
+      <c r="I29" s="13" t="n">
         <v>31</v>
       </c>
       <c r="J29" s="4" t="n">
         <v>5.21</v>
       </c>
+      <c r="K29" s="18" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C30" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D30" s="13" t="s">
-        <v>54</v>
+      <c r="A30" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>59</v>
       </c>
       <c r="E30" s="3" t="n">
         <f aca="false">SUM(F30:H30)</f>
@@ -1943,25 +2145,28 @@
       <c r="H30" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I30" s="12" t="n">
+      <c r="I30" s="13" t="n">
         <v>33</v>
       </c>
       <c r="J30" s="4" t="n">
         <v>4.761</v>
       </c>
+      <c r="K30" s="18" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B31" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C31" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D31" s="13" t="s">
-        <v>55</v>
+      <c r="A31" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>60</v>
       </c>
       <c r="E31" s="3" t="n">
         <f aca="false">SUM(F31:H31)</f>
@@ -1976,25 +2181,28 @@
       <c r="H31" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I31" s="12" t="n">
+      <c r="I31" s="13" t="n">
         <v>31</v>
       </c>
       <c r="J31" s="4" t="n">
         <v>14.408</v>
       </c>
+      <c r="K31" s="18" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C32" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="13" t="s">
-        <v>56</v>
+      <c r="A32" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>61</v>
       </c>
       <c r="E32" s="3" t="n">
         <f aca="false">SUM(F32:H32)</f>
@@ -2009,25 +2217,28 @@
       <c r="H32" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I32" s="12" t="n">
+      <c r="I32" s="13" t="n">
         <v>47</v>
       </c>
       <c r="J32" s="4" t="n">
         <v>20.704</v>
       </c>
+      <c r="K32" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D33" s="13" t="s">
-        <v>57</v>
+      <c r="A33" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>62</v>
       </c>
       <c r="E33" s="3" t="n">
         <f aca="false">SUM(F33:H33)</f>
@@ -2042,25 +2253,28 @@
       <c r="H33" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I33" s="12" t="n">
+      <c r="I33" s="13" t="n">
         <v>40</v>
       </c>
       <c r="J33" s="4" t="n">
         <v>19.677</v>
       </c>
+      <c r="K33" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D34" s="13" t="s">
-        <v>58</v>
+      <c r="A34" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>63</v>
       </c>
       <c r="E34" s="3" t="n">
         <f aca="false">SUM(F34:H34)</f>
@@ -2075,25 +2289,28 @@
       <c r="H34" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I34" s="12" t="n">
+      <c r="I34" s="13" t="n">
         <v>35</v>
       </c>
       <c r="J34" s="4" t="n">
         <v>2.548</v>
       </c>
+      <c r="K34" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D35" s="13" t="s">
-        <v>59</v>
+      <c r="A35" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>64</v>
       </c>
       <c r="E35" s="3" t="n">
         <f aca="false">SUM(F35:H35)</f>
@@ -2108,25 +2325,28 @@
       <c r="H35" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I35" s="12" t="n">
+      <c r="I35" s="13" t="n">
         <v>47</v>
       </c>
       <c r="J35" s="4" t="n">
         <v>18.884</v>
       </c>
+      <c r="K35" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C36" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D36" s="13" t="s">
-        <v>60</v>
+      <c r="A36" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B36" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>65</v>
       </c>
       <c r="E36" s="3" t="n">
         <f aca="false">SUM(F36:H36)</f>
@@ -2141,25 +2361,28 @@
       <c r="H36" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I36" s="12" t="n">
+      <c r="I36" s="13" t="n">
         <v>36</v>
       </c>
       <c r="J36" s="4" t="n">
         <v>1.397</v>
       </c>
+      <c r="K36" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C37" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D37" s="13" t="s">
-        <v>61</v>
+      <c r="A37" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>66</v>
       </c>
       <c r="E37" s="3" t="n">
         <f aca="false">SUM(F37:H37)</f>
@@ -2174,25 +2397,28 @@
       <c r="H37" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I37" s="12" t="n">
+      <c r="I37" s="13" t="n">
         <v>50</v>
       </c>
       <c r="J37" s="4" t="n">
         <v>1.371</v>
       </c>
+      <c r="K37" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B38" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C38" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D38" s="13" t="s">
-        <v>62</v>
+      <c r="A38" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>67</v>
       </c>
       <c r="E38" s="3" t="n">
         <f aca="false">SUM(F38:H38)</f>
@@ -2207,25 +2433,28 @@
       <c r="H38" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I38" s="12" t="n">
+      <c r="I38" s="13" t="n">
         <v>44</v>
       </c>
       <c r="J38" s="4" t="n">
         <v>104</v>
       </c>
+      <c r="K38" s="19" t="n">
+        <v>4.384</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B39" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C39" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D39" s="13" t="s">
-        <v>56</v>
+      <c r="A39" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B39" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>61</v>
       </c>
       <c r="E39" s="3" t="n">
         <f aca="false">SUM(F39:H39)</f>
@@ -2240,25 +2469,28 @@
       <c r="H39" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I39" s="12" t="n">
+      <c r="I39" s="13" t="n">
         <v>48</v>
       </c>
       <c r="J39" s="4" t="n">
         <v>29.6</v>
       </c>
+      <c r="K39" s="19" t="n">
+        <v>3.312</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C40" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D40" s="13" t="s">
-        <v>63</v>
+      <c r="A40" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B40" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>68</v>
       </c>
       <c r="E40" s="3" t="n">
         <f aca="false">SUM(F40:H40)</f>
@@ -2273,25 +2505,28 @@
       <c r="H40" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I40" s="12" t="n">
+      <c r="I40" s="13" t="n">
         <v>54</v>
       </c>
       <c r="J40" s="4" t="n">
         <v>69.5</v>
       </c>
+      <c r="K40" s="19" t="n">
+        <v>5.95599999999999</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B41" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C41" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D41" s="13" t="s">
-        <v>64</v>
+      <c r="A41" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B41" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>69</v>
       </c>
       <c r="E41" s="3" t="n">
         <f aca="false">SUM(F41:H41)</f>
@@ -2306,25 +2541,28 @@
       <c r="H41" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I41" s="12" t="n">
+      <c r="I41" s="13" t="n">
         <v>52</v>
       </c>
       <c r="J41" s="4" t="n">
         <v>17.4</v>
       </c>
+      <c r="K41" s="19" t="n">
+        <v>4.88</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B42" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C42" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D42" s="13" t="s">
-        <v>65</v>
+      <c r="A42" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B42" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>70</v>
       </c>
       <c r="E42" s="3" t="n">
         <f aca="false">SUM(F42:H42)</f>
@@ -2339,32 +2577,35 @@
       <c r="H42" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I42" s="12" t="n">
+      <c r="I42" s="13" t="n">
         <v>36</v>
       </c>
       <c r="J42" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="K42" s="19" t="n">
+        <v>8.97</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C43" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D43" s="13" t="s">
-        <v>66</v>
+      <c r="A43" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B43" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>68</v>
       </c>
       <c r="E43" s="3" t="n">
         <f aca="false">SUM(F43:H43)</f>
-        <v>49</v>
+        <v>11.2930826137372</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>49</v>
+        <v>11.2930826137372</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>0</v>
@@ -2372,32 +2613,35 @@
       <c r="H43" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I43" s="12" t="n">
-        <v>37</v>
+      <c r="I43" s="13" t="n">
+        <v>31</v>
       </c>
       <c r="J43" s="4" t="n">
-        <v>49</v>
+        <v>26</v>
+      </c>
+      <c r="K43" s="18" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B44" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C44" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D44" s="13" t="s">
-        <v>67</v>
+      <c r="A44" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B44" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C44" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D44" s="14" t="s">
+        <v>66</v>
       </c>
       <c r="E44" s="3" t="n">
         <f aca="false">SUM(F44:H44)</f>
-        <v>18.8</v>
+        <v>6</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>18.8</v>
+        <v>6</v>
       </c>
       <c r="G44" s="4" t="n">
         <v>0</v>
@@ -2405,32 +2649,35 @@
       <c r="H44" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I44" s="12" t="n">
-        <v>35</v>
+      <c r="I44" s="13" t="n">
+        <v>33</v>
       </c>
       <c r="J44" s="4" t="n">
-        <v>18.8</v>
+        <v>6</v>
+      </c>
+      <c r="K44" s="18" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B45" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C45" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D45" s="13" t="s">
-        <v>68</v>
+      <c r="A45" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B45" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D45" s="14" t="s">
+        <v>71</v>
       </c>
       <c r="E45" s="3" t="n">
         <f aca="false">SUM(F45:H45)</f>
-        <v>8.3</v>
+        <v>3</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>8.3</v>
+        <v>3</v>
       </c>
       <c r="G45" s="4" t="n">
         <v>0</v>
@@ -2438,32 +2685,35 @@
       <c r="H45" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I45" s="12" t="n">
-        <v>40</v>
+      <c r="I45" s="13" t="n">
+        <v>32</v>
       </c>
       <c r="J45" s="4" t="n">
-        <v>8.3</v>
+        <v>3</v>
+      </c>
+      <c r="K45" s="18" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B46" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C46" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D46" s="13" t="s">
-        <v>69</v>
+      <c r="A46" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B46" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C46" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D46" s="14" t="s">
+        <v>72</v>
       </c>
       <c r="E46" s="3" t="n">
         <f aca="false">SUM(F46:H46)</f>
-        <v>3</v>
+        <v>2.6914669995602</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>3</v>
+        <v>2.6914669995602</v>
       </c>
       <c r="G46" s="4" t="n">
         <v>0</v>
@@ -2471,32 +2721,35 @@
       <c r="H46" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I46" s="12" t="n">
-        <v>33</v>
+      <c r="I46" s="13" t="n">
+        <v>31</v>
       </c>
       <c r="J46" s="4" t="n">
-        <v>3</v>
+        <v>59</v>
+      </c>
+      <c r="K46" s="18" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B47" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C47" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D47" s="13" t="s">
-        <v>70</v>
+      <c r="A47" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B47" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C47" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D47" s="14" t="s">
+        <v>73</v>
       </c>
       <c r="E47" s="3" t="n">
         <f aca="false">SUM(F47:H47)</f>
-        <v>1</v>
+        <v>0.947886827981485</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>1</v>
+        <v>0.947886827981485</v>
       </c>
       <c r="G47" s="4" t="n">
         <v>0</v>
@@ -2504,32 +2757,35 @@
       <c r="H47" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I47" s="12" t="n">
-        <v>40</v>
+      <c r="I47" s="13" t="n">
+        <v>36</v>
       </c>
       <c r="J47" s="4" t="n">
-        <v>1</v>
+        <v>16</v>
+      </c>
+      <c r="K47" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B48" s="12" t="s">
+      <c r="A48" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B48" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C48" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C48" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D48" s="13" t="s">
-        <v>63</v>
+      <c r="D48" s="14" t="s">
+        <v>74</v>
       </c>
       <c r="E48" s="3" t="n">
         <f aca="false">SUM(F48:H48)</f>
-        <v>11.2930826137372</v>
+        <v>0.701721705388288</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>11.2930826137372</v>
+        <v>0.701721705388288</v>
       </c>
       <c r="G48" s="4" t="n">
         <v>0</v>
@@ -2537,32 +2793,35 @@
       <c r="H48" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I48" s="12" t="n">
-        <v>31</v>
+      <c r="I48" s="13" t="n">
+        <v>35</v>
       </c>
       <c r="J48" s="4" t="n">
-        <v>26</v>
+        <v>44</v>
+      </c>
+      <c r="K48" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B49" s="12" t="s">
+      <c r="A49" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B49" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C49" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C49" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D49" s="13" t="s">
-        <v>61</v>
+      <c r="D49" s="14" t="s">
+        <v>75</v>
       </c>
       <c r="E49" s="3" t="n">
         <f aca="false">SUM(F49:H49)</f>
-        <v>6</v>
+        <v>0.0258911233622709</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>6</v>
+        <v>0.0258911233622709</v>
       </c>
       <c r="G49" s="4" t="n">
         <v>0</v>
@@ -2570,32 +2829,35 @@
       <c r="H49" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I49" s="12" t="n">
-        <v>33</v>
+      <c r="I49" s="13" t="n">
+        <v>60</v>
       </c>
       <c r="J49" s="4" t="n">
-        <v>6</v>
+        <v>20</v>
+      </c>
+      <c r="K49" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B50" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C50" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D50" s="13" t="s">
-        <v>71</v>
+      <c r="A50" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C50" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D50" s="14" t="s">
+        <v>76</v>
       </c>
       <c r="E50" s="3" t="n">
         <f aca="false">SUM(F50:H50)</f>
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="G50" s="4" t="n">
         <v>0</v>
@@ -2603,32 +2865,35 @@
       <c r="H50" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I50" s="12" t="n">
-        <v>32</v>
+      <c r="I50" s="13" t="n">
+        <v>37</v>
       </c>
       <c r="J50" s="4" t="n">
-        <v>3</v>
+        <v>49</v>
+      </c>
+      <c r="K50" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B51" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C51" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D51" s="13" t="s">
-        <v>72</v>
+      <c r="A51" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B51" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C51" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D51" s="14" t="s">
+        <v>77</v>
       </c>
       <c r="E51" s="3" t="n">
         <f aca="false">SUM(F51:H51)</f>
-        <v>2.6914669995602</v>
+        <v>18.8</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>2.6914669995602</v>
+        <v>18.8</v>
       </c>
       <c r="G51" s="4" t="n">
         <v>0</v>
@@ -2636,32 +2901,35 @@
       <c r="H51" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I51" s="12" t="n">
-        <v>31</v>
+      <c r="I51" s="13" t="n">
+        <v>35</v>
       </c>
       <c r="J51" s="4" t="n">
-        <v>59</v>
+        <v>18.8</v>
+      </c>
+      <c r="K51" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B52" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C52" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D52" s="13" t="s">
-        <v>73</v>
+      <c r="A52" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B52" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C52" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D52" s="14" t="s">
+        <v>75</v>
       </c>
       <c r="E52" s="3" t="n">
         <f aca="false">SUM(F52:H52)</f>
-        <v>0.947886827981485</v>
+        <v>8.3</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>0.947886827981485</v>
+        <v>8.3</v>
       </c>
       <c r="G52" s="4" t="n">
         <v>0</v>
@@ -2669,32 +2937,35 @@
       <c r="H52" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I52" s="12" t="n">
-        <v>36</v>
+      <c r="I52" s="13" t="n">
+        <v>40</v>
       </c>
       <c r="J52" s="4" t="n">
+        <v>8.3</v>
+      </c>
+      <c r="K52" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B53" s="13" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B53" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C53" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D53" s="13" t="s">
-        <v>74</v>
+      <c r="C53" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D53" s="14" t="s">
+        <v>78</v>
       </c>
       <c r="E53" s="3" t="n">
         <f aca="false">SUM(F53:H53)</f>
-        <v>0.701721705388288</v>
+        <v>3</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>0.701721705388288</v>
+        <v>3</v>
       </c>
       <c r="G53" s="4" t="n">
         <v>0</v>
@@ -2702,32 +2973,35 @@
       <c r="H53" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I53" s="12" t="n">
-        <v>35</v>
+      <c r="I53" s="13" t="n">
+        <v>33</v>
       </c>
       <c r="J53" s="4" t="n">
-        <v>44</v>
+        <v>3</v>
+      </c>
+      <c r="K53" s="18" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B54" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C54" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D54" s="13" t="s">
-        <v>68</v>
+      <c r="A54" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B54" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C54" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D54" s="14" t="s">
+        <v>79</v>
       </c>
       <c r="E54" s="3" t="n">
         <f aca="false">SUM(F54:H54)</f>
-        <v>0.0258911233622709</v>
+        <v>1</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>0.0258911233622709</v>
+        <v>1</v>
       </c>
       <c r="G54" s="4" t="n">
         <v>0</v>
@@ -2735,11 +3009,14 @@
       <c r="H54" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I54" s="12" t="n">
-        <v>60</v>
+      <c r="I54" s="13" t="n">
+        <v>40</v>
       </c>
       <c r="J54" s="4" t="n">
-        <v>20</v>
+        <v>1</v>
+      </c>
+      <c r="K54" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2747,7 +3024,7 @@
       <c r="B55" s="6"/>
       <c r="C55" s="6"/>
       <c r="D55" s="6" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="E55" s="8" t="n">
         <f aca="false">SUBTOTAL(9,E5:E54)</f>
@@ -2770,39 +3047,45 @@
         <f aca="false">SUBTOTAL(9,J5:J54)</f>
         <v>881.056</v>
       </c>
+      <c r="K55" s="6"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="16" t="s">
-        <v>76</v>
+      <c r="A57" s="20" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="17" t="s">
-        <v>77</v>
+      <c r="A58" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="17" t="s">
-        <v>78</v>
+      <c r="A59" s="9" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="17" t="s">
-        <v>79</v>
+      <c r="A60" s="9" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="17" t="s">
-        <v>80</v>
+      <c r="A61" s="9" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="17" t="s">
-        <v>81</v>
+      <c r="A62" s="9" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="9" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J54"/>
+  <autoFilter ref="A4:K54"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>